<commit_message>
content: planilha trilingue (PT/EN/ES) dos 10 posts + pacote Exame
Adiciona versoes completas em EN e ES (nao so comentario) para os 10 posts
e o pacote Exame (email/social/whatsapp).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N1maUhe3cFZbTZXEjPto9a
</commit_message>
<xml_diff>
--- a/adfactory/content/terraventos-conteudos.xlsx
+++ b/adfactory/content/terraventos-conteudos.xlsx
@@ -60,12 +60,13 @@
     <col min="3" max="3" width="4" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="60" customWidth="1"/>
-    <col min="7" max="7" width="60" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="10" width="11" customWidth="1"/>
-    <col min="11" max="11" width="34" customWidth="1"/>
+    <col min="6" max="6" width="54" customWidth="1"/>
+    <col min="7" max="7" width="54" customWidth="1"/>
+    <col min="8" max="8" width="54" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="11" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -101,31 +102,36 @@
       </c>
       <c r="G1" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Comentário (EN)</t>
+          <t xml:space="preserve">Texto (EN)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Texto (ES)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Hashtags</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="2">
+      <c r="J1" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">CTA</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="2">
+      <c r="K1" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="2">
+      <c r="L1" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Observações</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="170" customHeight="1">
+    <row r="2" ht="200" customHeight="1">
       <c r="A2" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">FOIL-1</t>
@@ -161,31 +167,42 @@
       </c>
       <c r="G2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">🪽 The wind lifted — literally. It was beautiful to watch foil take over the Ceará sky this weekend, together with Instituto Ecoar. Athletes flying over the water, the community united, nature at the centre. Ceará isn't just the capital of wind — it's becoming the home of foil in Brazil. Tag someone who needs to see this fly. 👇</t>
+          <t xml:space="preserve">🪽 The wind lifted — literally.
+It was beautiful to watch foil take over the Ceará sky this weekend, together with Instituto Ecoar. 🌊
+Athletes flying over the water, the community united, nature at the centre. Ceará isn't just the capital of wind — it's becoming the home of foil in Brazil.
+Tag someone who needs to see this fly. 👇</t>
         </is>
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">🪽 El viento levantó — literalmente.
+Fue hermoso ver el foil apoderarse del cielo del litoral de Ceará este fin de semana, junto al Instituto Ecoar. 🌊
+Atletas volando sobre el agua, la comunidad reunida y la naturaleza en el centro de todo. Ceará no es solo la capital del viento — se está convirtiendo en la casa del foil en Brasil.
+Etiqueta a quien necesita ver esto volar. 👇</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#foil #wingfoil #kitefoil #Ceará #InstitutoEcoar #TerraVentos #litoralcearense #vento</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr" s="1">
+      <c r="J2" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Fala com a gente — link na bio.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Anexar mídia do evento (Google Drive). Citar @institutoecoar.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="170" customHeight="1">
+    <row r="3" ht="200" customHeight="1">
       <c r="A3" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">FOIL-2</t>
@@ -221,31 +238,42 @@
       </c>
       <c r="G3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Ever seen someone "fly" over the sea? 🪽 That's foil: a wing under the board that lifts the rider above the water — silent, light, almost magic. And there's no better stage for it than the Ceará wind. At the event with Instituto Ecoar it was exactly that: sea on one side, sky on the other, the rider between them. Which Ceará beach would you fly from? 🌬️</t>
+          <t xml:space="preserve">Ever seen someone "fly" over the sea? 🪽
+That's foil: a wing under the board that lifts the rider above the water — silent, light, almost magic. And there's no better stage for it than the Ceará wind.
+At the event with Instituto Ecoar it was exactly that: sea on one side, sky on the other, the rider between them.
+Which Ceará beach would you fly from? 🌬️</t>
         </is>
       </c>
       <c r="H3" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">¿Alguna vez viste a alguien "volar" sobre el mar? 🪽
+Eso es el foil: un ala bajo la tabla que eleva al rider por encima del agua — silencioso, ligero, casi mágico. Y no hay mejor escenario que el viento de Ceará.
+En el evento con el Instituto Ecoar fue exactamente así: el mar de un lado, el cielo del otro, y el rider entre los dos.
+¿Qué playa de Ceará elegirías para volar? 🌬️</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#foil #wingfoil #Ceará #InstitutoEcoar #TerraVentos #kite #vento</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr" s="1">
+      <c r="J3" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Comenta sua praia favorita.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Anexar mídia do evento (Google Drive). Citar @institutoecoar.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="170" customHeight="1">
+    <row r="4" ht="200" customHeight="1">
       <c r="A4" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">FOIL-3</t>
@@ -281,31 +309,42 @@
       </c>
       <c r="G4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Behind every flight, a community. 🤝 What stood out most at the foil event with Instituto Ecoar wasn't just the performance — it was the people. Riders from everywhere, the same wind, the same respect for the sea. That community is what makes the Ceará coast unique. Tell us in the comments: where are you from and where do you ride? 🌍</t>
+          <t xml:space="preserve">Behind every flight, a community. 🤝
+What stood out most at the foil event with Instituto Ecoar wasn't just the performance — it was the people. Riders from everywhere, the same wind, the same respect for the sea.
+That community is what makes the Ceará coast unique.
+Tell us in the comments: where are you from and where do you ride? 🌍</t>
         </is>
       </c>
       <c r="H4" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Detrás de cada vuelo, una comunidad. 🤝
+Lo que más marcó en el evento de foil con el Instituto Ecoar no fue solo el rendimiento — fue la gente. Riders de todas partes, el mismo viento, el mismo respeto por el mar.
+Esa comunidad es lo que hace único al litoral de Ceará.
+Cuéntanos en los comentarios: ¿de dónde eres y dónde navegas? 🌍</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#foilcommunity #wingfoil #Ceará #InstitutoEcoar #TerraVentos #kitesurf</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr" s="1">
+      <c r="J4" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Comenta de onde você é.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K4" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Anexar mídia do evento (Google Drive). Citar @institutoecoar.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="170" customHeight="1">
+    <row r="5" ht="200" customHeight="1">
       <c r="A5" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">FOIL-4</t>
@@ -340,31 +379,40 @@
       </c>
       <c r="G5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">The quietest sport on the sea is also one of the most conscious. 🌱 No motor, no noise, no trace — foil glides and leaves the ocean as it found it. That's why the partnership with Instituto Ecoar makes so much sense: protecting the coast that gives this sport life. Flying over the water is also a commitment to care for it. 🌊</t>
+          <t xml:space="preserve">The quietest sport on the sea is also one of the most conscious. 🌱
+No motor, no noise, no trace — foil glides and leaves the ocean as it found it. That's why the partnership with Instituto Ecoar makes so much sense: protecting the coast that gives this sport life.
+Flying over the water is also a commitment to care for it. 🌊</t>
         </is>
       </c>
       <c r="H5" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">El deporte más silencioso del mar también es uno de los más conscientes. 🌱
+Sin motor, sin ruido, sin estela — el foil se desliza dejando el océano como lo encontró. Por eso la alianza con el Instituto Ecoar tiene tanto sentido: preservar el litoral que da vida a este deporte.
+Volar sobre el agua es también un compromiso de cuidarla. 🌊</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#NavegarÉPreservar #foil #InstitutoEcoar #sustentabilidade #Ceará #TerraVentos</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr" s="1">
+      <c r="J5" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Marca quem ama o mar.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Anexar mídia do evento (Google Drive). Citar @institutoecoar.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="170" customHeight="1">
+    <row r="6" ht="200" customHeight="1">
       <c r="A6" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">FOIL-5</t>
@@ -399,31 +447,40 @@
       </c>
       <c r="G6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Remember this: Ceará will be known as one of the birthplaces of foil in Brazil. 🪽 The same wind that put Jericoacoara and Preá on the world map is now lifting a new generation of riders — and, with Instituto Ecoar, doing it consciously. When a sport grows on a coast, the coast grows with it. Those who arrive early fly higher. 😉</t>
+          <t xml:space="preserve">Remember this: Ceará will be known as one of the birthplaces of foil in Brazil. 🪽
+The same wind that put Jericoacoara and Preá on the world map is now lifting a new generation of riders — and, with Instituto Ecoar, doing it consciously.
+When a sport grows on a coast, the coast grows with it. Those who arrive early fly higher. 😉</t>
         </is>
       </c>
       <c r="H6" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Guarda este nombre: Ceará será recordado como una de las cunas del foil en Brasil. 🪽
+El mismo viento que puso a Jericoacoara y Preá en el mapa del mundo ahora eleva una nueva generación de riders — y, con el Instituto Ecoar, de forma consciente.
+Cuando un deporte crece en una costa, la costa crece con él. Quien llega temprano, vuela más alto. 😉</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#foil #Ceará #Jericoacoara #Preá #InstitutoEcoar #TerraVentos #vento</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr" s="1">
+      <c r="J6" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Bora conversar sobre viver perto do vento? Link na bio.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K6" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Anexar mídia do evento (Google Drive). Citar @institutoecoar.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="170" customHeight="1">
+    <row r="7" ht="200" customHeight="1">
       <c r="A7" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">TEMA-1</t>
@@ -458,31 +515,40 @@
       </c>
       <c r="G7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Bitupitá isn't the end of the map — it's the start of the Parnaíba Delta. 🌊 Ceará's largest mangrove, dunes like a pocket Lençóis and five rivers meeting the sea. One of Brazil's last untouched stretches of coast — and maybe the most special. Did you know this side of Ceará? 👇</t>
+          <t xml:space="preserve">Bitupitá isn't the end of the map — it's the start of the Parnaíba Delta. 🌊
+Ceará's largest mangrove, dunes like a pocket Lençóis and five rivers meeting the sea. One of Brazil's last untouched stretches of coast — and maybe the most special.
+Did you know this side of Ceará? 👇</t>
         </is>
       </c>
       <c r="H7" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Bitupitá no es el fin del mapa — es el comienzo del Delta del Parnaíba. 🌊
+El mayor manglar de Ceará, dunas que recuerdan a un mini Lençóis y el encuentro de cinco ríos con el mar. Uno de los últimos tramos vírgenes del litoral brasileño — y quizás el más especial.
+¿Conocías este lado de Ceará? 👇</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#Bitupitá #DeltaDoParnaíba #RotaDasEmoções #Ceará #TerraVentos #natureza</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr" s="1">
+      <c r="J7" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Leia no blog (link na bio).</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K7" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Baseado em bitupita-delta-fatos.md. Anexar foto/vídeo real (Drive/acervo).</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="170" customHeight="1">
+    <row r="8" ht="200" customHeight="1">
       <c r="A8" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">TEMA-2</t>
@@ -517,31 +583,40 @@
       </c>
       <c r="G8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">When big capital discovers a coast, it chases one thing: land. 📈 Megaprojects, international hotels and billions in investment are arriving on the Ceará coast. On the stretches still early in the curve — Bitupitá, Tatajuba, Preá — land is still within reach for those who come early. Before Jeri became Jeri, someone bought early.</t>
+          <t xml:space="preserve">When big capital discovers a coast, it chases one thing: land. 📈
+Megaprojects, international hotels and billions in investment are arriving on the Ceará coast. On the stretches still early in the curve — Bitupitá, Tatajuba, Preá — land is still within reach for those who come early.
+Before Jeri became Jeri, someone bought early.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Cuando el gran capital descubre una costa, va detrás de una cosa: tierra. 📈
+Megaproyectos, hoteles internacionales y miles de millones en inversión están llegando al litoral de Ceará. En los tramos que aún están al inicio de la curva — Bitupitá, Tatajuba, Preá — la tierra todavía está al alcance de quien llega temprano.
+Antes de que Jeri fuera Jeri, alguien compró temprano.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#investimento #Ceará #terreno #litoralcearense #TerraVentos #Bitupitá #Tatajuba</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr" s="1">
+      <c r="J8" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Vamos conversar? Link na bio.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K8" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Sem promessa de retorno. Anexar foto/vídeo real (Drive/acervo).</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="170" customHeight="1">
+    <row r="9" ht="200" customHeight="1">
       <c r="A9" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">TEMA-3</t>
@@ -576,31 +651,40 @@
       </c>
       <c r="G9" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Six months of wind, June to December. The rest of the year is yours to live. 🪁 Preá, Jericoacoara, Cumbuco — Ceará is one of the best kite destinations on earth. Now imagine your place on the sand right in the middle of it. What's your favourite spot? 🌬️</t>
+          <t xml:space="preserve">Six months of wind, June to December. The rest of the year is yours to live. 🪁
+Preá, Jericoacoara, Cumbuco — Ceará is one of the best kite destinations on earth. Now imagine your place on the sand right in the middle of it.
+What's your favourite spot? 🌬️</t>
         </is>
       </c>
       <c r="H9" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Seis meses de viento, de junio a diciembre. El resto del año, es tuyo para vivir. 🪁
+Preá, Jericoacoara, Cumbuco — Ceará es uno de los mejores destinos de kite del planeta. Ahora imagina tener tu lugar en la arena justo en el medio de todo.
+¿Cuál es tu spot favorito? 🌬️</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#kitesurf #Preá #Jericoacoara #Cumbuco #Ceará #TerraVentos #vento</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr" s="1">
+      <c r="J9" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Comenta seu spot.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K9" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Respeita a trava factual (jun–dez). Anexar foto/vídeo real (Drive/acervo).</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="170" customHeight="1">
+    <row r="10" ht="200" customHeight="1">
       <c r="A10" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">TEMA-4</t>
@@ -635,31 +719,40 @@
       </c>
       <c r="G10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">What if your kite spot had your name on the deed? 🌍 More and more foreigners are finding that investing on the Ceará coast can also be the first step to living in Brazil. The right land, legal security, and a life with the wind at your back. We'll show you the way — in the right order. 📩</t>
+          <t xml:space="preserve">What if your kite spot had your name on the deed? 🌍
+More and more foreigners are finding that investing on the Ceará coast can also be the first step to living in Brazil. The right land, legal security, and a life with the wind at your back.
+We'll show you the way — in the right order. 📩</t>
         </is>
       </c>
       <c r="H10" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">¿Y si tu spot de kite tuviera tu nombre en la escritura? 🌍
+Cada vez más extranjeros descubren que invertir en el litoral de Ceará puede ser también el primer paso para vivir en Brasil. La tierra correcta, seguridad jurídica y una vida con el viento a favor.
+Te mostramos el camino — en el orden correcto. 📩</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#goldenvisa #Brazil #Ceará #kitesurf #realestate #TerraVentos #investinbrazil</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr" s="1">
+      <c r="J10" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Fala com a gente — link na bio.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K10" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Anexar foto/vídeo real (Drive/acervo).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="170" customHeight="1">
+    <row r="11" ht="200" customHeight="1">
       <c r="A11" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">TEMA-5</t>
@@ -694,31 +787,40 @@
       </c>
       <c r="G11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">A coast only stays beautiful if someone cares for it. 🌱 That's why we support initiatives like Instituto Ecoar: protecting the beaches, dunes and sea that make Ceará what it is. Investing here is also a commitment to this place. Tag someone who loves the Ceará coast. 🌊</t>
+          <t xml:space="preserve">A coast only stays beautiful if someone cares for it. 🌱
+That's why we support initiatives like Instituto Ecoar: protecting the beaches, dunes and sea that make Ceará what it is. Investing here is also a commitment to this place.
+Tag someone who loves the Ceará coast. 🌊</t>
         </is>
       </c>
       <c r="H11" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">Un litoral solo sigue siendo hermoso si alguien lo cuida. 🌱
+Por eso apoyamos iniciativas como el Instituto Ecoar: preservar las playas, las dunas y el mar que hacen de Ceará lo que es. Invertir aquí es también comprometerse con este lugar.
+Etiqueta a quien ama el litoral de Ceará. 🌊</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#InstitutoEcoar #sustentabilidade #Ceará #litoralcearense #TerraVentos #NavegarÉPreservar</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr" s="1">
+      <c r="J11" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Marca quem ama o litoral.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K11" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Citar @institutoecoar. Anexar foto/vídeo real (Drive/acervo).</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="170" customHeight="1">
+    <row r="12" ht="200" customHeight="1">
       <c r="A12" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">EXAM-1</t>
@@ -765,31 +867,46 @@
       </c>
       <c r="G12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">SUBJECT: Capital is arriving on the Ceará coast — and land is still within reach. Hi [name], Exame reported on a family that sold their land in Ceará for a billion-real project. It's not isolated — it's the symptom of a bigger move: luxury megaprojects in Preá minutes from Jericoacoara airport, global hotel flags (Anantara) announced for 2026, tens of billions across the Northeast, and wind sports drawing buyers worldwide. When big capital finds a coast, it chases land — and land is what we curate in Bitupitá, Tatajuba and Preá, with clean title. Want to talk, no strings? Message us on WhatsApp. Terra Ventos — Invest with the wind at your back.</t>
+          <t xml:space="preserve">SUBJECT: Capital is arriving on the Ceará coast — and land is still within reach.
+Hi [name],
+Exame reported on a family that sold their land in Ceará for a billion-real project. It's not isolated — it's the symptom of a bigger move: luxury megaprojects in Preá minutes from Jericoacoara airport, global hotel flags (Anantara) announced for 2026, tens of billions across the Northeast, and wind sports drawing buyers worldwide.
+When big capital finds a coast, it chases land — and land is what we curate in Bitupitá, Tatajuba and Preá, with clean title.
+Want to talk, no strings? Message us on WhatsApp.
+Terra Ventos — Invest with the wind at your back. Source: Exame.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">ASUNTO: El capital está llegando al litoral de Ceará — y la tierra aún es accesible.
+Hola [nombre],
+¿Lo viste? Exame contó la historia de una familia que vendió su terreno en Ceará para un proyecto multimillonario. No es un caso aislado: megaproyectos de lujo en Preá a minutos del aeropuerto de Jericoacoara, banderas hoteleras globales (Anantara) anunciadas para 2026, decenas de miles de millones en el Nordeste y el turismo deportivo atrayendo compradores de todo el mundo.
+Cuando el gran capital descubre una costa, va detrás de la tierra — y eso es lo que cuidamos contigo en Bitupitá, Tatajuba y Preá, con documentación limpia.
+¿Hablamos, sin compromiso? Escríbenos por WhatsApp.
+Terra Ventos — Invierte con el viento a favor. Fuente: Exame.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr" s="1">
+      <c r="J12" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Ver oportunidades / WhatsApp</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K12" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Confirmar se pode citar a Exame. Não foi possível ler o corpo do artigo (bloqueio). Sem promessa de retorno.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="170" customHeight="1">
+    <row r="13" ht="200" customHeight="1">
       <c r="A13" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">EXAM-2</t>
@@ -828,31 +945,48 @@
       </c>
       <c r="G13" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">🌊 R$30 billion. That's how hungry capital is for the Ceará coast right now. Exame reported on a family that sold their land for a billion-real project — but the message is bigger than one sale: luxury megaprojects in Preá minutes from Jeri airport, international hotel flags arriving in 2026, and wind, kite and foil turning beaches into sought-after addresses. When big money finds a coast, it chases land. And land — in Bitupitá, Tatajuba, Preá — is still within reach for those who arrive early. Before Jeri became Jeri, someone bought early. 👀</t>
+          <t xml:space="preserve">🌊 R$30 billion. That's how hungry capital is for the Ceará coast right now.
+Exame reported on a family that sold their land for a billion-real project — but the message is bigger than one sale:
+📈 Luxury megaprojects in Preá, minutes from Jeri airport.
+🏨 International hotel flags arriving in 2026.
+💨 Wind, kite and foil turning beaches into sought-after addresses.
+When big money finds a coast, it chases land. And land — in Bitupitá, Tatajuba, Preá — is still within reach for those who arrive early.
+Before Jeri became Jeri, someone bought early. 👀</t>
         </is>
       </c>
       <c r="H13" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">🌊 R$30 mil millones. Ese es el apetito que tiene el capital por el litoral de Ceará ahora.
+Exame contó la historia de una familia que vendió su terreno para un proyecto multimillonario. Pero el mensaje es más grande que una venta:
+📈 Megaproyectos de lujo en Preá, a minutos del aeropuerto de Jeri.
+🏨 Banderas hoteleras internacionales llegando en 2026.
+💨 El viento, el kite y el foil convirtiendo playas en direcciones codiciadas.
+Cuando el gran dinero descubre una costa, va detrás de la tierra. Y la tierra — en Bitupitá, Tatajuba, Preá — todavía está al alcance de quien llega temprano.
+Antes de que Jeri fuera Jeri, alguien compró temprano. 👀</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">#Ceará #Jericoacoara #Preá #Bitupitá #Tatajuba #investimentoimobiliário #litoralcearense #RotaDasEmoções</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr" s="1">
+      <c r="J13" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Fala com a gente — link na bio.</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K13" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">Fonte: Exame. Confirmar citação nominal.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="170" customHeight="1">
+    <row r="14" ht="200" customHeight="1">
       <c r="A14" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">EXAM-3</t>
@@ -889,25 +1023,38 @@
       </c>
       <c r="G14" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Hi [name]! 🌊 Did you see Exame's story about the family that sold their land in Ceará for a billion-real project? It's the sign of a move we follow closely: capital pouring into the Ceará coast — megaprojects in Preá, international hotels arriving in 2026, kite and foil drawing the world. Good news: on the stretches still early in the curve (Bitupitá, Tatajuba, Preá), land is still affordable. Want me to show you 2–3 beachfront opportunities that fit this moment? No strings. 🙌 — Terra Ventos</t>
+          <t xml:space="preserve">Hi [name]! 🌊 Did you see Exame's story about the family that sold their land in Ceará for a billion-real project?
+It's the sign of a move we follow closely: capital pouring into the Ceará coast — megaprojects in Preá, international hotels arriving in 2026, kite and foil drawing the world.
+Good news: on the stretches still early in the curve (Bitupitá, Tatajuba, Preá), land is still affordable.
+Want me to show you 2–3 beachfront opportunities that fit this moment? No strings. 🙌
+— Terra Ventos</t>
         </is>
       </c>
       <c r="H14" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">¡Hola [nombre]! 🌊 ¿Viste la nota de Exame sobre la familia que vendió su terreno en Ceará para un proyecto multimillonario?
+Es la señal de un movimiento que seguimos de cerca: el capital entrando fuerte en el litoral de Ceará — megaproyectos en Preá, hoteles internacionales llegando en 2026, el kite y el foil atrayendo al mundo.
+La buena noticia: en los tramos que aún están al inicio de la curva (Bitupitá, Tatajuba, Preá), la tierra todavía es accesible.
+¿Quieres que te muestre 2 o 3 oportunidades frente al mar que tienen sentido para este momento? Sin compromiso. 🙌
+— Terra Ventos</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr" s="1">
+      <c r="J14" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Resposta no WhatsApp</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">rascunho</t>
-        </is>
-      </c>
       <c r="K14" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">rascunho</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Personalizar [nome]. Fonte: Exame.</t>
         </is>

</xml_diff>